<commit_message>
upgrade protoc to 3.30.2
</commit_message>
<xml_diff>
--- a/src/Monster.xlsx
+++ b/src/Monster.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28730"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Shark\ExcelToBytes\src\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{935A0117-1DB5-4A79-87A6-8CF7F3D2DF24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="24225" windowHeight="12540"/>
+    <workbookView xWindow="32811" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monster" sheetId="1" r:id="rId1"/>
@@ -15,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="61">
   <si>
     <t>optional</t>
   </si>
@@ -186,19 +192,29 @@
   </si>
   <si>
     <t>10002-15</t>
+  </si>
+  <si>
+    <t>c</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>cs</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>ClientOnly</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>只在Client生成</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
-  <fonts count="21">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -213,151 +229,21 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
+      <sz val="9"/>
       <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="10"/>
       <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
-  <fills count="35">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -376,194 +262,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -586,255 +286,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -850,59 +308,24 @@
     <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="货币[0]" xfId="1" builtinId="7"/>
-    <cellStyle name="20% - 强调文字颜色 3" xfId="2" builtinId="38"/>
-    <cellStyle name="输入" xfId="3" builtinId="20"/>
-    <cellStyle name="货币" xfId="4" builtinId="4"/>
-    <cellStyle name="千位分隔[0]" xfId="5" builtinId="6"/>
-    <cellStyle name="40% - 强调文字颜色 3" xfId="6" builtinId="39"/>
-    <cellStyle name="差" xfId="7" builtinId="27"/>
-    <cellStyle name="千位分隔" xfId="8" builtinId="3"/>
-    <cellStyle name="60% - 强调文字颜色 3" xfId="9" builtinId="40"/>
-    <cellStyle name="超链接" xfId="10" builtinId="8"/>
-    <cellStyle name="百分比" xfId="11" builtinId="5"/>
-    <cellStyle name="已访问的超链接" xfId="12" builtinId="9"/>
-    <cellStyle name="注释" xfId="13" builtinId="10"/>
-    <cellStyle name="60% - 强调文字颜色 2" xfId="14" builtinId="36"/>
-    <cellStyle name="标题 4" xfId="15" builtinId="19"/>
-    <cellStyle name="警告文本" xfId="16" builtinId="11"/>
-    <cellStyle name="标题" xfId="17" builtinId="15"/>
-    <cellStyle name="解释性文本" xfId="18" builtinId="53"/>
-    <cellStyle name="标题 1" xfId="19" builtinId="16"/>
-    <cellStyle name="标题 2" xfId="20" builtinId="17"/>
-    <cellStyle name="60% - 强调文字颜色 1" xfId="21" builtinId="32"/>
-    <cellStyle name="标题 3" xfId="22" builtinId="18"/>
-    <cellStyle name="60% - 强调文字颜色 4" xfId="23" builtinId="44"/>
-    <cellStyle name="输出" xfId="24" builtinId="21"/>
-    <cellStyle name="计算" xfId="25" builtinId="22"/>
-    <cellStyle name="检查单元格" xfId="26" builtinId="23"/>
-    <cellStyle name="20% - 强调文字颜色 6" xfId="27" builtinId="50"/>
-    <cellStyle name="强调文字颜色 2" xfId="28" builtinId="33"/>
-    <cellStyle name="链接单元格" xfId="29" builtinId="24"/>
-    <cellStyle name="汇总" xfId="30" builtinId="25"/>
-    <cellStyle name="好" xfId="31" builtinId="26"/>
-    <cellStyle name="适中" xfId="32" builtinId="28"/>
-    <cellStyle name="20% - 强调文字颜色 5" xfId="33" builtinId="46"/>
-    <cellStyle name="强调文字颜色 1" xfId="34" builtinId="29"/>
-    <cellStyle name="20% - 强调文字颜色 1" xfId="35" builtinId="30"/>
-    <cellStyle name="40% - 强调文字颜色 1" xfId="36" builtinId="31"/>
-    <cellStyle name="20% - 强调文字颜色 2" xfId="37" builtinId="34"/>
-    <cellStyle name="40% - 强调文字颜色 2" xfId="38" builtinId="35"/>
-    <cellStyle name="强调文字颜色 3" xfId="39" builtinId="37"/>
-    <cellStyle name="强调文字颜色 4" xfId="40" builtinId="41"/>
-    <cellStyle name="20% - 强调文字颜色 4" xfId="41" builtinId="42"/>
-    <cellStyle name="40% - 强调文字颜色 4" xfId="42" builtinId="43"/>
-    <cellStyle name="强调文字颜色 5" xfId="43" builtinId="45"/>
-    <cellStyle name="40% - 强调文字颜色 5" xfId="44" builtinId="47"/>
-    <cellStyle name="60% - 强调文字颜色 5" xfId="45" builtinId="48"/>
-    <cellStyle name="强调文字颜色 6" xfId="46" builtinId="49"/>
-    <cellStyle name="40% - 强调文字颜色 6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor indexed="10"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -915,6 +338,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1201,21 +627,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:I17"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.15" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="8" width="9" style="1"/>
-    <col min="9" max="9" width="17.125" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="9" style="1"/>
+    <col min="9" max="9" width="17.15234375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="16.15234375" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1243,8 +670,11 @@
       <c r="I1" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -1272,8 +702,11 @@
       <c r="I2" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" spans="1:9">
+      <c r="J2" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>8</v>
       </c>
@@ -1301,8 +734,11 @@
       <c r="I3" s="4" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:9">
+      <c r="J3" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>8</v>
       </c>
@@ -1330,8 +766,11 @@
       <c r="I4" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:9">
+      <c r="J4" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>25</v>
       </c>
@@ -1356,11 +795,14 @@
       <c r="H5" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I5" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
+      <c r="I5" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
@@ -1388,8 +830,11 @@
       <c r="I6" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="7" spans="1:9">
+      <c r="J6" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>10002</v>
       </c>
@@ -1417,8 +862,11 @@
       <c r="I7" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="8" spans="1:9">
+      <c r="J7" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>10003</v>
       </c>
@@ -1446,8 +894,11 @@
       <c r="I8" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="9" spans="1:9">
+      <c r="J8" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>10004</v>
       </c>
@@ -1475,8 +926,11 @@
       <c r="I9" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="10" spans="1:9">
+      <c r="J9" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>10005</v>
       </c>
@@ -1504,8 +958,11 @@
       <c r="I10" s="1" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="11" spans="1:9">
+      <c r="J10" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10006</v>
       </c>
@@ -1533,8 +990,11 @@
       <c r="I11" s="1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="12" spans="1:9">
+      <c r="J11" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>10007</v>
       </c>
@@ -1562,8 +1022,11 @@
       <c r="I12" s="1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="13" spans="1:9">
+      <c r="J12" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>10008</v>
       </c>
@@ -1591,8 +1054,11 @@
       <c r="I13" s="1" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="14" spans="1:9">
+      <c r="J13" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>10009</v>
       </c>
@@ -1620,8 +1086,11 @@
       <c r="I14" s="1" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="15" spans="1:9">
+      <c r="J14" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>10010</v>
       </c>
@@ -1649,8 +1118,11 @@
       <c r="I15" s="1" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="16" spans="1:9">
+      <c r="J15" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>10011</v>
       </c>
@@ -1678,8 +1150,11 @@
       <c r="I16" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="17" spans="1:9">
+      <c r="J16" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>10012</v>
       </c>
@@ -1707,111 +1182,33 @@
       <c r="I17" s="1" t="s">
         <v>56</v>
       </c>
+      <c r="J17" s="1">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A1">
-    <cfRule type="cellIs" dxfId="0" priority="21" stopIfTrue="1" operator="notEqual">
+  <phoneticPr fontId="2" type="noConversion"/>
+  <conditionalFormatting sqref="A1:J1">
+    <cfRule type="cellIs" dxfId="1" priority="1" stopIfTrue="1" operator="notEqual">
       <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B1">
-    <cfRule type="cellIs" dxfId="0" priority="18" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C1">
-    <cfRule type="cellIs" dxfId="0" priority="11" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D1">
-    <cfRule type="cellIs" dxfId="0" priority="10" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E1">
-    <cfRule type="cellIs" dxfId="0" priority="9" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F1">
-    <cfRule type="cellIs" dxfId="0" priority="8" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G1">
-    <cfRule type="cellIs" dxfId="0" priority="5" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H1">
-    <cfRule type="cellIs" dxfId="0" priority="3" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I1">
-    <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A4">
-    <cfRule type="cellIs" dxfId="0" priority="22" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B4">
-    <cfRule type="cellIs" dxfId="0" priority="17" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C4">
-    <cfRule type="cellIs" dxfId="0" priority="16" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D4">
-    <cfRule type="cellIs" dxfId="0" priority="15" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E4">
-    <cfRule type="cellIs" dxfId="0" priority="14" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F4">
-    <cfRule type="cellIs" dxfId="0" priority="13" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G4">
-    <cfRule type="cellIs" dxfId="0" priority="6" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H4">
-    <cfRule type="cellIs" dxfId="0" priority="4" stopIfTrue="1" operator="notEqual">
-      <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I4">
+  <conditionalFormatting sqref="A4:J4">
     <cfRule type="cellIs" dxfId="0" priority="2" stopIfTrue="1" operator="notEqual">
       <formula>INDIRECT("Dummy_for_Comparison1!"&amp;ADDRESS(ROW(),COLUMN()))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.15" x14ac:dyDescent="0.3"/>
   <sheetData/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>